<commit_message>
Need to fit recent data to really know whats what
</commit_message>
<xml_diff>
--- a/BeatnotePostHotCell/Jun05,2026/Fit_ResultJun5.xlsx
+++ b/BeatnotePostHotCell/Jun05,2026/Fit_ResultJun5.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostHotCell\Jun05,2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476A84CA-FA54-40AE-B1A9-04FE272AAFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D7131B-6F84-4684-AD2B-4FC78B53BB25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D9E101C5-8284-4B59-8B1C-2AD2D5F2FDD3}"/>
   </bookViews>
   <sheets>
-    <sheet name="456" sheetId="1" r:id="rId1"/>
-    <sheet name="894" sheetId="2" r:id="rId2"/>
+    <sheet name="894" sheetId="2" r:id="rId1"/>
+    <sheet name="456" sheetId="1" r:id="rId2"/>
     <sheet name="AbsCoef" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="13">
   <si>
     <t>Date</t>
   </si>
@@ -78,12 +78,6 @@
   </si>
   <si>
     <t>Jun05,2026+3-03-33PM</t>
-  </si>
-  <si>
-    <t>Jun05,2026+3-44-13PM</t>
-  </si>
-  <si>
-    <t>Jun05,2026+5-40-35PM</t>
   </si>
 </sst>
 </file>
@@ -460,6 +454,162 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40C5617D-2BBC-4C21-ADC4-3687FEC8C6E3}">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="42.75">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1">
+        <v>8.5895120122534792</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1.32175631481448</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-1.47660814776098E-3</v>
+      </c>
+      <c r="E2" s="1">
+        <v>2.0461989026218399</v>
+      </c>
+      <c r="F2" s="1">
+        <v>61.015977316476103</v>
+      </c>
+      <c r="G2" s="1">
+        <v>2.2873007307343098E-3</v>
+      </c>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" ht="42.75">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1">
+        <v>8.6524212475503699</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1.3220594476084</v>
+      </c>
+      <c r="D3" s="1">
+        <v>-1.37090013722952E-3</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1.7954604424870899</v>
+      </c>
+      <c r="F3" s="1">
+        <v>61.015845170582203</v>
+      </c>
+      <c r="G3" s="1">
+        <v>2.2873004957281199E-3</v>
+      </c>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" ht="42.75">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1">
+        <v>8.2927304597387206</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1.3225766972684201</v>
+      </c>
+      <c r="D4" s="1">
+        <v>-9.1354722651605799E-4</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2.0435771205192301</v>
+      </c>
+      <c r="F4" s="1">
+        <v>62.033611955772002</v>
+      </c>
+      <c r="G4" s="1">
+        <v>2.2873004957024599E-3</v>
+      </c>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" ht="42.75">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="1">
+        <v>8.4368095561837997</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1.3230781346721601</v>
+      </c>
+      <c r="D5" s="1">
+        <v>-1.3458462333547599E-3</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1.9955264747896599</v>
+      </c>
+      <c r="F5" s="1">
+        <v>63.092636759922698</v>
+      </c>
+      <c r="G5" s="1">
+        <v>3.4359424898629202E-3</v>
+      </c>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" ht="42.75">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1">
+        <v>8.6554109919161206</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1.31634191469888</v>
+      </c>
+      <c r="D6" s="1">
+        <v>-4.4180379946506999E-4</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1.7942664653895199</v>
+      </c>
+      <c r="F6" s="1">
+        <v>61.127234720085902</v>
+      </c>
+      <c r="G6" s="1">
+        <v>2.2873004957028398E-3</v>
+      </c>
+      <c r="H6" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011646E0-737D-49FA-A2CA-7848F848076B}">
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -495,7 +645,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="1">
-        <v>0.14198189433295499</v>
+        <v>0.110683626430072</v>
       </c>
       <c r="C2" s="1">
         <v>1.4720893886703099</v>
@@ -507,13 +657,13 @@
         <v>-1.64279899450385E-4</v>
       </c>
       <c r="F2" s="1">
-        <v>2.1446542829716</v>
+        <v>2.0834835314285498</v>
       </c>
       <c r="G2" s="1">
-        <v>61.117610369704899</v>
+        <v>61.219535066680699</v>
       </c>
       <c r="H2" s="1">
-        <v>6.0598065389552605E-4</v>
+        <v>1.1280764960870499E-3</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="42.75">
@@ -521,7 +671,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="1">
-        <v>0.14200693706074399</v>
+        <v>0.110618484823125</v>
       </c>
       <c r="C3" s="1">
         <v>1.4736233725494301</v>
@@ -533,13 +683,13 @@
         <v>-5.9615449363946401E-5</v>
       </c>
       <c r="F3" s="1">
-        <v>1.9001195748405799</v>
+        <v>1.8389533784904799</v>
       </c>
       <c r="G3" s="1">
-        <v>63.032265965089103</v>
+        <v>63.034434937411199</v>
       </c>
       <c r="H3" s="1">
-        <v>1.0391347847576401E-3</v>
+        <v>1.1342108032927501E-3</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="42.75">
@@ -547,7 +697,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="1">
-        <v>0.13879302222888601</v>
+        <v>0.108110401129387</v>
       </c>
       <c r="C4" s="1">
         <v>1.47443200713404</v>
@@ -559,13 +709,13 @@
         <v>-1.15744481920728E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>2.4014522578758499</v>
+        <v>2.3402905470054001</v>
       </c>
       <c r="G4" s="1">
-        <v>62.621278196769701</v>
+        <v>62.623173152241201</v>
       </c>
       <c r="H4" s="1">
-        <v>1.07708648791815E-3</v>
+        <v>1.1417462572662501E-3</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="42.75">
@@ -573,7 +723,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="1">
-        <v>0.14134057599559999</v>
+        <v>0.110098201353416</v>
       </c>
       <c r="C5" s="1">
         <v>1.47339477827734</v>
@@ -585,13 +735,13 @@
         <v>-1.07866087506238E-4</v>
       </c>
       <c r="F5" s="1">
-        <v>1.36000748390472</v>
+        <v>1.2988524057553501</v>
       </c>
       <c r="G5" s="1">
-        <v>63.084424122596197</v>
+        <v>63.084085972996199</v>
       </c>
       <c r="H5" s="1">
-        <v>1.0504388815699901E-3</v>
+        <v>1.14466496785816E-3</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="42.75">
@@ -599,7 +749,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="1">
-        <v>0.14287369952523299</v>
+        <v>0.111279548853152</v>
       </c>
       <c r="C6" s="1">
         <v>1.4735825089765799</v>
@@ -611,222 +761,34 @@
         <v>-3.0439945155011898E-4</v>
       </c>
       <c r="F6" s="1">
-        <v>1.1445913004167201</v>
+        <v>1.0834292453218199</v>
       </c>
       <c r="G6" s="1">
-        <v>61.259100724127897</v>
+        <v>61.1729315751911</v>
       </c>
       <c r="H6" s="1">
-        <v>5.7874152140768398E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="42.75">
-      <c r="A7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1">
-        <v>0.14058451279890199</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1.47277606233849</v>
-      </c>
-      <c r="D7" s="1">
-        <v>1.0380759954383399E-3</v>
-      </c>
-      <c r="E7" s="1">
-        <v>-1.3827494162170701E-4</v>
-      </c>
-      <c r="F7" s="1">
-        <v>1.14530027036071</v>
-      </c>
-      <c r="G7" s="1">
-        <v>61.127889610880402</v>
-      </c>
-      <c r="H7" s="1">
-        <v>5.8008235598823899E-4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="42.75">
-      <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1">
-        <v>0.142306901322892</v>
-      </c>
-      <c r="C8" s="1">
-        <v>1.47414356157587</v>
-      </c>
-      <c r="D8" s="2">
-        <v>4.7666632358515602E-5</v>
-      </c>
-      <c r="E8" s="1">
-        <v>-1.3370878868840301E-4</v>
-      </c>
-      <c r="F8" s="1">
-        <v>3.3958231526152698</v>
-      </c>
-      <c r="G8" s="1">
-        <v>63.141018630769999</v>
-      </c>
-      <c r="H8" s="1">
-        <v>1.128340315432E-3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40C5617D-2BBC-4C21-ADC4-3687FEC8C6E3}">
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="42.75">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1">
-        <v>8.5895120122534792</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1.32175631481448</v>
-      </c>
-      <c r="D2" s="1">
-        <v>-1.47660814776098E-3</v>
-      </c>
-      <c r="E2" s="1">
-        <v>2.0461989026218399</v>
-      </c>
-      <c r="F2" s="1">
-        <v>61.015977316476103</v>
-      </c>
-      <c r="G2" s="1">
-        <v>2.2873007307343098E-3</v>
-      </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" ht="42.75">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1">
-        <v>8.6524212475503699</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1.3220594476084</v>
-      </c>
-      <c r="D3" s="1">
-        <v>-1.37090013722952E-3</v>
-      </c>
-      <c r="E3" s="1">
-        <v>1.7954604424870899</v>
-      </c>
-      <c r="F3" s="1">
-        <v>61.015845170582203</v>
-      </c>
-      <c r="G3" s="1">
-        <v>2.2873004957281199E-3</v>
-      </c>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" ht="42.75">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1">
-        <v>8.2927304597387206</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1.3225766972684201</v>
-      </c>
-      <c r="D4" s="1">
-        <v>-9.1354722651605799E-4</v>
-      </c>
-      <c r="E4" s="1">
-        <v>2.0435771205192301</v>
-      </c>
-      <c r="F4" s="1">
-        <v>62.033611955772002</v>
-      </c>
-      <c r="G4" s="1">
-        <v>2.2873004957024599E-3</v>
-      </c>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" ht="42.75">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1">
-        <v>8.4368095561837997</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1.3230781346721601</v>
-      </c>
-      <c r="D5" s="1">
-        <v>-1.3458462333547599E-3</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1.9955264747896599</v>
-      </c>
-      <c r="F5" s="1">
-        <v>63.092636759922698</v>
-      </c>
-      <c r="G5" s="1">
-        <v>3.4359424898629202E-3</v>
-      </c>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" ht="42.75">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1">
-        <v>8.6554109919161206</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1.31634191469888</v>
-      </c>
-      <c r="D6" s="1">
-        <v>-4.4180379946506999E-4</v>
-      </c>
-      <c r="E6" s="1">
-        <v>1.7942664653895199</v>
-      </c>
-      <c r="F6" s="1">
-        <v>61.127234720085902</v>
-      </c>
-      <c r="G6" s="1">
-        <v>2.2873004957028398E-3</v>
-      </c>
-      <c r="H6" s="1"/>
+        <v>6.5140429823798602E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -835,10 +797,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF8CB368-1F4F-4C65-B86B-93EC676CB77B}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -846,80 +808,62 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="42.75">
+    <row r="2" spans="1:3" ht="42.75">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="1">
-        <v>0.14198189433295499</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1">
         <v>8.5895120122534792</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="42.75">
+      <c r="C2" s="1">
+        <v>0.110683626430072</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="42.75">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="1">
-        <v>0.14200693706074399</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="1">
         <v>8.6524212475503699</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="42.75">
+      <c r="C3" s="1">
+        <v>0.110618484823125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="42.75">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="1">
-        <v>0.13879302222888601</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="1">
         <v>8.2927304597387206</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="42.75">
+      <c r="C4" s="1">
+        <v>0.108110401129387</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="42.75">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="1">
-        <v>0.14134057599559999</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="1">
         <v>8.4368095561837997</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="42.75">
+      <c r="C5" s="1">
+        <v>0.110098201353416</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="42.75">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="1">
-        <v>0.14287369952523299</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="1">
         <v>8.6554109919161206</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.111279548853152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>